<commit_message>
full deep test SDC-IC bolts
</commit_message>
<xml_diff>
--- a/tests/designcodes/res/M12_bolt.xlsx
+++ b/tests/designcodes/res/M12_bolt.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="R:\AC_ResultsDB\Pietro\Alberto\EPP01 BOLOMETERS\BoltAssessment\geometries\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DATA\laghida\Documents\GitLab\cassy\tests\designcodes\res\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{644226E6-CC1F-46B1-919E-12E8EC2EC782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{421FF4F3-C3AF-434B-B47D-242FDAAC8E06}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5670" yWindow="1710" windowWidth="21600" windowHeight="11385" xr2:uid="{F09436F1-1F29-42A5-B1F9-53A78950820F}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{F09436F1-1F29-42A5-B1F9-53A78950820F}"/>
   </bookViews>
   <sheets>
     <sheet name="Bolt Data" sheetId="1" r:id="rId1"/>
@@ -1432,7 +1432,7 @@
         <v>19</v>
       </c>
       <c r="C9" s="31">
-        <v>12.5</v>
+        <v>10.11</v>
       </c>
       <c r="D9" s="5" t="s">
         <v>7</v>
@@ -1453,7 +1453,7 @@
         <v>35</v>
       </c>
       <c r="C10" s="30">
-        <v>14.615</v>
+        <v>14.05</v>
       </c>
       <c r="D10" s="5" t="s">
         <v>7</v>
@@ -1474,7 +1474,7 @@
         <v>21</v>
       </c>
       <c r="C11" s="31">
-        <v>16</v>
+        <v>13.22</v>
       </c>
       <c r="D11" s="5" t="s">
         <v>7</v>
@@ -1516,7 +1516,7 @@
         <v>43</v>
       </c>
       <c r="C13" s="31">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="D13" s="5" t="s">
         <v>7</v>
@@ -1752,6 +1752,15 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="71e126cb-1963-4e7b-b13a-15d2f64f78e9">
@@ -1760,15 +1769,6 @@
     <TaxCatchAll xmlns="f41f4605-e15c-4135-bd96-d3970596b173" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -2001,6 +2001,14 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F460EF5-1FE2-485A-B28D-6307C5242F38}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B53875E3-DFDB-4F02-8AAC-AEAA1E089733}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
@@ -2009,14 +2017,6 @@
     <ds:schemaRef ds:uri="cfb58fdf-baa4-49ab-9b9a-8c103073e122"/>
     <ds:schemaRef ds:uri="71e126cb-1963-4e7b-b13a-15d2f64f78e9"/>
     <ds:schemaRef ds:uri="f41f4605-e15c-4135-bd96-d3970596b173"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{7F460EF5-1FE2-485A-B28D-6307C5242F38}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>